<commit_message>
update publications and outreach
</commit_message>
<xml_diff>
--- a/content.xlsx
+++ b/content.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8120"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8115"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>title</t>
   </si>
@@ -57,9 +57,6 @@
     <t>https://essd.copernicus.org/articles/16/2625/2024/</t>
   </si>
   <si>
-    <t>indicators-climate-change.png</t>
-  </si>
-  <si>
     <t>Indicators of global climate change 2023</t>
   </si>
   <si>
@@ -115,6 +112,18 @@
   </si>
   <si>
     <t>A current list of countries that have peaked in GHG emissions and reduced for more than 10 years.</t>
+  </si>
+  <si>
+    <t>indicators-climate-change-2023.png</t>
+  </si>
+  <si>
+    <t>Indicators of global climate change 2024</t>
+  </si>
+  <si>
+    <t>indicators-climate-change-2024.png</t>
+  </si>
+  <si>
+    <t>https://essd.copernicus.org/preprints/essd-2025-250/</t>
   </si>
 </sst>
 </file>
@@ -443,10 +452,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -457,10 +466,10 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -471,97 +480,111 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C7" r:id="rId1"/>
-    <hyperlink ref="C4" r:id="rId2"/>
+    <hyperlink ref="C8" r:id="rId1"/>
+    <hyperlink ref="C5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>